<commit_message>
feat: align configurator with strict Excel 1:1 rules
Port configurator inputs and calculations to worksheet-driven rule IDs with formula reconciliation by cell references, and persist schema-versioned draft snapshots for reliable regression checks.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/WEB/added/Новая таблица для расчета.xlsx
+++ b/WEB/added/Новая таблица для расчета.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CH-CRM\WEB\added\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C2FFDF-49C9-475D-82E4-A61EB0F32F76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F354B04-B8F4-4F8D-B81F-7FE9A512E1CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{E985C3AD-E5E2-7B43-93DF-C13AA55BC74F}"/>
+    <workbookView xWindow="-25635" yWindow="-465" windowWidth="19860" windowHeight="15135" activeTab="2" xr2:uid="{E985C3AD-E5E2-7B43-93DF-C13AA55BC74F}"/>
   </bookViews>
   <sheets>
     <sheet name="Таблица для заполнения" sheetId="2" r:id="rId1"/>
@@ -30,6 +30,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -1357,37 +1360,79 @@
     <xf numFmtId="44" fontId="11" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1415,48 +1460,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1783,15 +1786,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="99" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="101"/>
+      <c r="B1" s="99"/>
       <c r="C1" s="40"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="102"/>
-      <c r="B2" s="102"/>
+      <c r="A2" s="100"/>
+      <c r="B2" s="100"/>
       <c r="C2" s="1" t="s">
         <v>77</v>
       </c>
@@ -1800,328 +1803,362 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="97" t="s">
+      <c r="A3" s="96" t="s">
         <v>87</v>
       </c>
-      <c r="B3" s="97"/>
+      <c r="B3" s="96"/>
       <c r="C3" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="6"/>
+      <c r="D3" s="6">
+        <v>120</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="97" t="s">
+      <c r="A4" s="96" t="s">
         <v>65</v>
       </c>
-      <c r="B4" s="97"/>
+      <c r="B4" s="96"/>
       <c r="C4" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="6"/>
+      <c r="D4" s="6">
+        <v>90</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="97" t="s">
+      <c r="A5" s="96" t="s">
         <v>66</v>
       </c>
-      <c r="B5" s="97"/>
+      <c r="B5" s="96"/>
       <c r="C5" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D5" s="6"/>
+      <c r="D5" s="6">
+        <v>2.7</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="98"/>
-      <c r="B6" s="99"/>
+      <c r="A6" s="97"/>
+      <c r="B6" s="98"/>
       <c r="C6" s="15"/>
       <c r="D6" s="6"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="98" t="s">
+      <c r="A7" s="97" t="s">
         <v>69</v>
       </c>
-      <c r="B7" s="99"/>
+      <c r="B7" s="98"/>
       <c r="C7" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="D7" s="13"/>
+      <c r="D7" s="13">
+        <v>110</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="98" t="s">
+      <c r="A8" s="97" t="s">
         <v>70</v>
       </c>
-      <c r="B8" s="99"/>
+      <c r="B8" s="98"/>
       <c r="C8" s="15" t="s">
         <v>78</v>
       </c>
       <c r="D8" s="13"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="98" t="s">
+      <c r="A9" s="97" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="99"/>
+      <c r="B9" s="98"/>
       <c r="C9" s="15" t="s">
         <v>78</v>
       </c>
       <c r="D9" s="13"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="98" t="s">
+      <c r="A10" s="97" t="s">
         <v>72</v>
       </c>
-      <c r="B10" s="99"/>
+      <c r="B10" s="98"/>
       <c r="C10" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="D10" s="13"/>
+      <c r="D10" s="13">
+        <v>100</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="98" t="s">
+      <c r="A11" s="97" t="s">
         <v>73</v>
       </c>
-      <c r="B11" s="99"/>
+      <c r="B11" s="98"/>
       <c r="C11" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="D11" s="13"/>
+      <c r="D11" s="13">
+        <v>10</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="98"/>
-      <c r="B12" s="99"/>
+      <c r="A12" s="97"/>
+      <c r="B12" s="98"/>
       <c r="C12" s="15"/>
       <c r="D12" s="6"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="98"/>
-      <c r="B13" s="99"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="98"/>
       <c r="C13" s="15"/>
       <c r="D13" s="6"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="98" t="s">
+      <c r="A14" s="97" t="s">
         <v>136</v>
       </c>
-      <c r="B14" s="99"/>
+      <c r="B14" s="98"/>
       <c r="C14" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="D14" s="23"/>
+      <c r="D14" s="23">
+        <v>200</v>
+      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="98"/>
-      <c r="B15" s="99"/>
+      <c r="A15" s="97"/>
+      <c r="B15" s="98"/>
       <c r="C15" s="15"/>
       <c r="D15" s="6"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="98"/>
-      <c r="B16" s="99"/>
+      <c r="A16" s="97"/>
+      <c r="B16" s="98"/>
       <c r="C16" s="15"/>
       <c r="D16" s="6"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="97" t="s">
+      <c r="A17" s="96" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="97"/>
+      <c r="B17" s="96"/>
       <c r="C17" s="6" t="s">
         <v>60</v>
       </c>
       <c r="D17" s="89"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="97" t="s">
+      <c r="A18" s="96" t="s">
         <v>67</v>
       </c>
-      <c r="B18" s="97"/>
+      <c r="B18" s="96"/>
       <c r="C18" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="89"/>
+      <c r="D18" s="89">
+        <v>150</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="97"/>
-      <c r="B19" s="97"/>
+      <c r="A19" s="96"/>
+      <c r="B19" s="96"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="97" t="s">
+      <c r="A20" s="96" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="97"/>
+      <c r="B20" s="96"/>
       <c r="C20" s="6" t="s">
         <v>60</v>
       </c>
       <c r="D20" s="6"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="97" t="s">
+      <c r="A21" s="96" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="97"/>
+      <c r="B21" s="96"/>
       <c r="C21" s="6" t="s">
         <v>60</v>
       </c>
       <c r="D21" s="6"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="97" t="s">
+      <c r="A22" s="96" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="97"/>
+      <c r="B22" s="96"/>
       <c r="C22" s="6" t="s">
         <v>60</v>
       </c>
       <c r="D22" s="6"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="97" t="s">
+      <c r="A23" s="96" t="s">
         <v>31</v>
       </c>
-      <c r="B23" s="97"/>
+      <c r="B23" s="96"/>
       <c r="C23" s="6" t="s">
         <v>60</v>
       </c>
       <c r="D23" s="6"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="97" t="s">
+      <c r="A24" s="96" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="97"/>
+      <c r="B24" s="96"/>
       <c r="C24" s="6" t="s">
         <v>60</v>
       </c>
       <c r="D24" s="6"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="97" t="s">
+      <c r="A25" s="96" t="s">
         <v>74</v>
       </c>
-      <c r="B25" s="97"/>
+      <c r="B25" s="96"/>
       <c r="C25" s="6" t="s">
         <v>60</v>
       </c>
       <c r="D25" s="6"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="97"/>
-      <c r="B26" s="97"/>
+      <c r="A26" s="96"/>
+      <c r="B26" s="96"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="97" t="s">
+      <c r="A27" s="96" t="s">
         <v>75</v>
       </c>
-      <c r="B27" s="97"/>
+      <c r="B27" s="96"/>
       <c r="C27" s="6" t="s">
         <v>78</v>
       </c>
       <c r="D27" s="6"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="97" t="s">
+      <c r="A28" s="96" t="s">
         <v>76</v>
       </c>
-      <c r="B28" s="97"/>
+      <c r="B28" s="96"/>
       <c r="C28" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D28" s="6"/>
+      <c r="D28" s="6">
+        <v>120</v>
+      </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="97"/>
-      <c r="B29" s="97"/>
+      <c r="A29" s="96"/>
+      <c r="B29" s="96"/>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="97" t="s">
+      <c r="A30" s="96" t="s">
         <v>80</v>
       </c>
-      <c r="B30" s="97"/>
+      <c r="B30" s="96"/>
       <c r="C30" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D30" s="6"/>
+      <c r="D30" s="6">
+        <v>5</v>
+      </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="97" t="s">
+      <c r="A31" s="96" t="s">
         <v>40</v>
       </c>
-      <c r="B31" s="97"/>
+      <c r="B31" s="96"/>
       <c r="C31" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D31" s="6"/>
+      <c r="D31" s="6">
+        <v>50000</v>
+      </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="97" t="s">
+      <c r="A32" s="96" t="s">
         <v>81</v>
       </c>
-      <c r="B32" s="97"/>
+      <c r="B32" s="96"/>
       <c r="C32" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D32" s="6"/>
+      <c r="D32" s="6">
+        <v>50000</v>
+      </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="97" t="s">
+      <c r="A33" s="96" t="s">
         <v>83</v>
       </c>
-      <c r="B33" s="97"/>
+      <c r="B33" s="96"/>
       <c r="C33" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D33" s="6"/>
+      <c r="D33" s="6">
+        <v>8</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="97" t="s">
+      <c r="A34" s="96" t="s">
         <v>84</v>
       </c>
-      <c r="B34" s="97"/>
+      <c r="B34" s="96"/>
       <c r="C34" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D34" s="6"/>
+      <c r="D34" s="6">
+        <v>120000</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="97" t="s">
+      <c r="A35" s="96" t="s">
         <v>88</v>
       </c>
-      <c r="B35" s="97"/>
+      <c r="B35" s="96"/>
       <c r="C35" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D35" s="6"/>
+      <c r="D35" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="36" spans="1:5" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="97" t="s">
+      <c r="A36" s="96" t="s">
         <v>86</v>
       </c>
-      <c r="B36" s="97"/>
+      <c r="B36" s="96"/>
       <c r="C36" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D36" s="6"/>
+      <c r="D36" s="6">
+        <v>30000</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="98" t="s">
+      <c r="A37" s="97" t="s">
         <v>85</v>
       </c>
-      <c r="B37" s="99"/>
+      <c r="B37" s="98"/>
       <c r="C37" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D37" s="6"/>
+      <c r="D37" s="6">
+        <v>1</v>
+      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="97" t="s">
+      <c r="A38" s="96" t="s">
         <v>110</v>
       </c>
-      <c r="B38" s="97"/>
+      <c r="B38" s="96"/>
       <c r="C38" s="39"/>
       <c r="D38" s="90" t="s">
         <v>127</v>
@@ -2129,59 +2166,77 @@
       <c r="E38" s="56"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="97"/>
-      <c r="B39" s="97"/>
+      <c r="A39" s="96"/>
+      <c r="B39" s="96"/>
       <c r="C39" s="39"/>
       <c r="D39" s="6"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="100"/>
-      <c r="B40" s="100"/>
+      <c r="A40" s="101"/>
+      <c r="B40" s="101"/>
       <c r="C40" s="39"/>
       <c r="D40" s="6"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="97"/>
-      <c r="B41" s="97"/>
+      <c r="A41" s="96"/>
+      <c r="B41" s="96"/>
       <c r="C41" s="39"/>
       <c r="D41" s="6"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="97"/>
-      <c r="B42" s="97"/>
+      <c r="A42" s="96"/>
+      <c r="B42" s="96"/>
       <c r="C42" s="39"/>
       <c r="D42" s="6"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="97"/>
-      <c r="B43" s="97"/>
+      <c r="A43" s="96"/>
+      <c r="B43" s="96"/>
       <c r="C43" s="39"/>
       <c r="D43" s="6"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="97"/>
-      <c r="B44" s="97"/>
+      <c r="A44" s="96"/>
+      <c r="B44" s="96"/>
       <c r="C44" s="39"/>
       <c r="D44" s="6"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="97"/>
-      <c r="B45" s="97"/>
+      <c r="A45" s="96"/>
+      <c r="B45" s="96"/>
       <c r="C45" s="39"/>
       <c r="D45" s="6"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="96"/>
-      <c r="B46" s="96"/>
+      <c r="A46" s="102"/>
+      <c r="B46" s="102"/>
     </row>
   </sheetData>
   <mergeCells count="46">
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A34:B34"/>
@@ -2198,30 +2253,12 @@
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -2259,14 +2296,14 @@
       <c r="E1" s="48" t="s">
         <v>107</v>
       </c>
-      <c r="G1" s="103" t="s">
+      <c r="G1" s="104" t="s">
         <v>112</v>
       </c>
-      <c r="H1" s="103"/>
-      <c r="I1" s="103"/>
-      <c r="J1" s="103"/>
-      <c r="K1" s="103"/>
-      <c r="L1" s="103"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="104"/>
+      <c r="K1" s="104"/>
+      <c r="L1" s="104"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="45" t="s">
@@ -2285,11 +2322,11 @@
         <f t="shared" ref="E2:E23" si="0">B2*D2</f>
         <v>11000</v>
       </c>
-      <c r="G2" s="104" t="s">
+      <c r="G2" s="103" t="s">
         <v>113</v>
       </c>
-      <c r="H2" s="104"/>
-      <c r="I2" s="104"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
       <c r="J2" s="5" t="s">
         <v>4</v>
       </c>
@@ -2317,11 +2354,11 @@
         <f t="shared" si="0"/>
         <v>60000</v>
       </c>
-      <c r="G3" s="97" t="s">
+      <c r="G3" s="96" t="s">
         <v>114</v>
       </c>
-      <c r="H3" s="97"/>
-      <c r="I3" s="97"/>
+      <c r="H3" s="96"/>
+      <c r="I3" s="96"/>
       <c r="J3" s="6">
         <v>1</v>
       </c>
@@ -2348,11 +2385,11 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G4" s="97" t="s">
+      <c r="G4" s="96" t="s">
         <v>115</v>
       </c>
-      <c r="H4" s="97"/>
-      <c r="I4" s="97"/>
+      <c r="H4" s="96"/>
+      <c r="I4" s="96"/>
       <c r="J4" s="6">
         <v>1</v>
       </c>
@@ -2381,11 +2418,11 @@
         <f t="shared" si="0"/>
         <v>29000</v>
       </c>
-      <c r="G5" s="97" t="s">
+      <c r="G5" s="96" t="s">
         <v>121</v>
       </c>
-      <c r="H5" s="97"/>
-      <c r="I5" s="97"/>
+      <c r="H5" s="96"/>
+      <c r="I5" s="96"/>
       <c r="J5" s="6">
         <v>1</v>
       </c>
@@ -2412,11 +2449,11 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G6" s="97" t="s">
+      <c r="G6" s="96" t="s">
         <v>122</v>
       </c>
-      <c r="H6" s="97"/>
-      <c r="I6" s="97"/>
+      <c r="H6" s="96"/>
+      <c r="I6" s="96"/>
       <c r="J6" s="6">
         <v>1</v>
       </c>
@@ -2443,11 +2480,11 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G7" s="97" t="s">
+      <c r="G7" s="96" t="s">
         <v>117</v>
       </c>
-      <c r="H7" s="97"/>
-      <c r="I7" s="97"/>
+      <c r="H7" s="96"/>
+      <c r="I7" s="96"/>
       <c r="J7" s="6">
         <v>1</v>
       </c>
@@ -2476,11 +2513,11 @@
         <f t="shared" si="0"/>
         <v>12000</v>
       </c>
-      <c r="G8" s="97" t="s">
+      <c r="G8" s="96" t="s">
         <v>118</v>
       </c>
-      <c r="H8" s="97"/>
-      <c r="I8" s="97"/>
+      <c r="H8" s="96"/>
+      <c r="I8" s="96"/>
       <c r="J8" s="6">
         <v>1</v>
       </c>
@@ -2509,11 +2546,11 @@
         <f t="shared" si="0"/>
         <v>10000</v>
       </c>
-      <c r="G9" s="97" t="s">
+      <c r="G9" s="96" t="s">
         <v>119</v>
       </c>
-      <c r="H9" s="97"/>
-      <c r="I9" s="97"/>
+      <c r="H9" s="96"/>
+      <c r="I9" s="96"/>
       <c r="J9" s="6">
         <v>1</v>
       </c>
@@ -2542,11 +2579,11 @@
         <f t="shared" si="0"/>
         <v>7000</v>
       </c>
-      <c r="G10" s="97" t="s">
+      <c r="G10" s="96" t="s">
         <v>120</v>
       </c>
-      <c r="H10" s="97"/>
-      <c r="I10" s="97"/>
+      <c r="H10" s="96"/>
+      <c r="I10" s="96"/>
       <c r="J10" s="6">
         <v>1</v>
       </c>
@@ -2575,11 +2612,11 @@
         <f t="shared" si="0"/>
         <v>4500</v>
       </c>
-      <c r="G11" s="97" t="s">
+      <c r="G11" s="96" t="s">
         <v>137</v>
       </c>
-      <c r="H11" s="97"/>
-      <c r="I11" s="97"/>
+      <c r="H11" s="96"/>
+      <c r="I11" s="96"/>
       <c r="J11" s="6">
         <v>1</v>
       </c>
@@ -2608,11 +2645,11 @@
         <f t="shared" si="0"/>
         <v>1500</v>
       </c>
-      <c r="G12" s="97" t="s">
+      <c r="G12" s="96" t="s">
         <v>123</v>
       </c>
-      <c r="H12" s="97"/>
-      <c r="I12" s="97"/>
+      <c r="H12" s="96"/>
+      <c r="I12" s="96"/>
       <c r="J12" s="6"/>
       <c r="K12" s="51">
         <v>7000</v>
@@ -2639,11 +2676,11 @@
         <f t="shared" si="0"/>
         <v>850</v>
       </c>
-      <c r="G13" s="97" t="s">
+      <c r="G13" s="96" t="s">
         <v>124</v>
       </c>
-      <c r="H13" s="97"/>
-      <c r="I13" s="97"/>
+      <c r="H13" s="96"/>
+      <c r="I13" s="96"/>
       <c r="J13" s="6"/>
       <c r="K13" s="51">
         <v>7000</v>
@@ -2670,11 +2707,11 @@
         <f t="shared" si="0"/>
         <v>650</v>
       </c>
-      <c r="G14" s="97" t="s">
+      <c r="G14" s="96" t="s">
         <v>129</v>
       </c>
-      <c r="H14" s="97"/>
-      <c r="I14" s="97"/>
+      <c r="H14" s="96"/>
+      <c r="I14" s="96"/>
       <c r="J14" s="6"/>
       <c r="K14" s="51">
         <v>7000</v>
@@ -2699,11 +2736,11 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G15" s="97" t="s">
+      <c r="G15" s="96" t="s">
         <v>140</v>
       </c>
-      <c r="H15" s="97"/>
-      <c r="I15" s="97"/>
+      <c r="H15" s="96"/>
+      <c r="I15" s="96"/>
       <c r="J15" s="6">
         <v>1</v>
       </c>
@@ -2732,11 +2769,11 @@
         <f t="shared" si="0"/>
         <v>20000</v>
       </c>
-      <c r="G16" s="97" t="s">
+      <c r="G16" s="96" t="s">
         <v>142</v>
       </c>
-      <c r="H16" s="97"/>
-      <c r="I16" s="97"/>
+      <c r="H16" s="96"/>
+      <c r="I16" s="96"/>
       <c r="J16" s="6"/>
       <c r="K16" s="51">
         <v>10000</v>
@@ -2761,11 +2798,11 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G17" s="97" t="s">
+      <c r="G17" s="96" t="s">
         <v>125</v>
       </c>
-      <c r="H17" s="97"/>
-      <c r="I17" s="97"/>
+      <c r="H17" s="96"/>
+      <c r="I17" s="96"/>
       <c r="J17" s="6">
         <f>SUM(J3:J16)</f>
         <v>10</v>
@@ -2896,6 +2933,16 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="G1:L1"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="G10:I10"/>
     <mergeCell ref="G11:I11"/>
     <mergeCell ref="G12:I12"/>
     <mergeCell ref="G2:I2"/>
@@ -2903,16 +2950,6 @@
     <mergeCell ref="G4:I4"/>
     <mergeCell ref="G5:I5"/>
     <mergeCell ref="G6:I6"/>
-    <mergeCell ref="G1:L1"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="G17:I17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3694,21 +3731,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="107" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="109" t="s">
+      <c r="A1" s="121" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="123" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="111">
+      <c r="C1" s="125">
         <f>'Таблица для заполнения'!D3</f>
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="108"/>
-      <c r="B2" s="110"/>
-      <c r="C2" s="112"/>
+      <c r="A2" s="122"/>
+      <c r="B2" s="124"/>
+      <c r="C2" s="126"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -3738,10 +3775,10 @@
       <c r="I3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="113" t="s">
+      <c r="J3" s="127" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="113"/>
+      <c r="K3" s="127"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
@@ -3752,7 +3789,7 @@
       </c>
       <c r="C4" s="7">
         <f>C1</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="3"/>
@@ -3762,14 +3799,14 @@
       <c r="G4" s="3"/>
       <c r="H4" s="78">
         <f>C4*F4</f>
-        <v>0</v>
+        <v>60000</v>
       </c>
       <c r="I4" s="78">
         <f>(D4+F4)*C4</f>
-        <v>0</v>
-      </c>
-      <c r="J4" s="114"/>
-      <c r="K4" s="115"/>
+        <v>60000</v>
+      </c>
+      <c r="J4" s="128"/>
+      <c r="K4" s="129"/>
     </row>
     <row r="5" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
@@ -3780,26 +3817,26 @@
       </c>
       <c r="C5" s="5">
         <f>'Таблица для заполнения'!D7</f>
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="D5" s="95">
         <v>3360</v>
       </c>
       <c r="E5" s="51">
         <f>C5*D5</f>
-        <v>0</v>
+        <v>369600</v>
       </c>
       <c r="F5" s="57">
         <v>950</v>
       </c>
       <c r="G5" s="51">
         <f>C5*F5</f>
-        <v>0</v>
+        <v>104500</v>
       </c>
       <c r="H5" s="78"/>
       <c r="I5" s="78">
         <f>(D5+F5)*C5</f>
-        <v>0</v>
+        <v>474100</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="10"/>
@@ -3834,13 +3871,13 @@
         <f>(D6+F6)*C6</f>
         <v>0</v>
       </c>
-      <c r="J6" s="97"/>
-      <c r="K6" s="97"/>
+      <c r="J6" s="96"/>
+      <c r="K6" s="96"/>
       <c r="M6" s="11"/>
-      <c r="N6" s="105" t="s">
+      <c r="N6" s="118" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="106"/>
+      <c r="O6" s="109"/>
     </row>
     <row r="7" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
@@ -3872,8 +3909,8 @@
         <f t="shared" ref="I7:I42" si="2">(D7+F7)*C7</f>
         <v>0</v>
       </c>
-      <c r="J7" s="97"/>
-      <c r="K7" s="97"/>
+      <c r="J7" s="96"/>
+      <c r="K7" s="96"/>
     </row>
     <row r="8" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
@@ -3884,34 +3921,34 @@
       </c>
       <c r="C8" s="6">
         <f>'Таблица для заполнения'!D10</f>
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D8" s="57">
         <v>2200</v>
       </c>
       <c r="E8" s="51">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>220000</v>
       </c>
       <c r="F8" s="57">
         <v>600</v>
       </c>
       <c r="G8" s="51">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>60000</v>
       </c>
       <c r="H8" s="78"/>
       <c r="I8" s="78">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J8" s="97"/>
-      <c r="K8" s="97"/>
+        <v>280000</v>
+      </c>
+      <c r="J8" s="96"/>
+      <c r="K8" s="96"/>
       <c r="M8" s="12"/>
-      <c r="N8" s="105" t="s">
+      <c r="N8" s="118" t="s">
         <v>19</v>
       </c>
-      <c r="O8" s="106"/>
+      <c r="O8" s="109"/>
     </row>
     <row r="9" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
@@ -3922,14 +3959,14 @@
       </c>
       <c r="C9" s="13">
         <f>'Таблица для заполнения'!D11</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D9" s="57">
         <v>9570</v>
       </c>
       <c r="E9" s="65">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>95700</v>
       </c>
       <c r="F9" s="57">
         <v>4000</v>
@@ -3937,14 +3974,14 @@
       <c r="G9" s="65"/>
       <c r="H9" s="79">
         <f>C9*F9</f>
-        <v>0</v>
+        <v>40000</v>
       </c>
       <c r="I9" s="79">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J9" s="116"/>
-      <c r="K9" s="116"/>
+        <v>135700</v>
+      </c>
+      <c r="J9" s="110"/>
+      <c r="K9" s="110"/>
     </row>
     <row r="10" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
@@ -3976,13 +4013,13 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J10" s="97"/>
-      <c r="K10" s="97"/>
+      <c r="J10" s="96"/>
+      <c r="K10" s="96"/>
       <c r="M10" s="14"/>
-      <c r="N10" s="105" t="s">
+      <c r="N10" s="118" t="s">
         <v>22</v>
       </c>
-      <c r="O10" s="106"/>
+      <c r="O10" s="109"/>
     </row>
     <row r="11" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
@@ -3993,29 +4030,29 @@
       </c>
       <c r="C11" s="6">
         <f>'Таблица для заполнения'!D14*('Таблица для заполнения'!D5+0.95)</f>
-        <v>0</v>
+        <v>730.00000000000011</v>
       </c>
       <c r="D11" s="57">
         <v>2830</v>
       </c>
       <c r="E11" s="51">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2065900.0000000002</v>
       </c>
       <c r="F11" s="57">
         <v>1200</v>
       </c>
       <c r="G11" s="51">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>876000.00000000012</v>
       </c>
       <c r="H11" s="78"/>
       <c r="I11" s="78">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J11" s="98"/>
-      <c r="K11" s="99"/>
+        <v>2941900.0000000005</v>
+      </c>
+      <c r="J11" s="97"/>
+      <c r="K11" s="98"/>
       <c r="M11" s="16"/>
     </row>
     <row r="12" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -4027,34 +4064,34 @@
       </c>
       <c r="C12" s="6">
         <f>'Таблица для заполнения'!D14*('Таблица для заполнения'!D5+0.15)</f>
-        <v>0</v>
+        <v>570</v>
       </c>
       <c r="D12" s="57">
         <v>2050</v>
       </c>
       <c r="E12" s="51">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1168500</v>
       </c>
       <c r="F12" s="57">
         <v>600</v>
       </c>
       <c r="G12" s="51">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>342000</v>
       </c>
       <c r="H12" s="78"/>
       <c r="I12" s="78">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J12" s="97"/>
-      <c r="K12" s="97"/>
+        <v>1510500</v>
+      </c>
+      <c r="J12" s="96"/>
+      <c r="K12" s="96"/>
       <c r="M12" s="17"/>
-      <c r="N12" s="105" t="s">
+      <c r="N12" s="118" t="s">
         <v>25</v>
       </c>
-      <c r="O12" s="106"/>
+      <c r="O12" s="109"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
@@ -4086,8 +4123,8 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J13" s="97"/>
-      <c r="K13" s="97"/>
+      <c r="J13" s="96"/>
+      <c r="K13" s="96"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
@@ -4098,29 +4135,29 @@
       </c>
       <c r="C14" s="6">
         <f>'Таблица для заполнения'!D18*('Таблица для заполнения'!D5+0.15)</f>
-        <v>0</v>
+        <v>427.5</v>
       </c>
       <c r="D14" s="57">
         <v>1410</v>
       </c>
       <c r="E14" s="51">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>602775</v>
       </c>
       <c r="F14" s="57">
         <v>600</v>
       </c>
       <c r="G14" s="51">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>256500</v>
       </c>
       <c r="H14" s="78"/>
       <c r="I14" s="78">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J14" s="97"/>
-      <c r="K14" s="97"/>
+        <v>859275</v>
+      </c>
+      <c r="J14" s="96"/>
+      <c r="K14" s="96"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
@@ -4152,8 +4189,8 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J15" s="97"/>
-      <c r="K15" s="97"/>
+      <c r="J15" s="96"/>
+      <c r="K15" s="96"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
@@ -4185,8 +4222,8 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J16" s="98"/>
-      <c r="K16" s="99"/>
+      <c r="J16" s="97"/>
+      <c r="K16" s="98"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
@@ -4218,8 +4255,8 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J17" s="98"/>
-      <c r="K17" s="99"/>
+      <c r="J17" s="97"/>
+      <c r="K17" s="98"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
@@ -4317,8 +4354,8 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J20" s="97"/>
-      <c r="K20" s="97"/>
+      <c r="J20" s="96"/>
+      <c r="K20" s="96"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
@@ -4329,29 +4366,29 @@
       </c>
       <c r="C21" s="6">
         <f>'Таблица для заполнения'!D28</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D21" s="57">
         <v>7580</v>
       </c>
       <c r="E21" s="51">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>909600</v>
       </c>
       <c r="F21" s="57">
         <v>1600</v>
       </c>
       <c r="G21" s="51">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>192000</v>
       </c>
       <c r="H21" s="78"/>
       <c r="I21" s="78">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J21" s="97"/>
-      <c r="K21" s="97"/>
+        <v>1101600</v>
+      </c>
+      <c r="J21" s="96"/>
+      <c r="K21" s="96"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
@@ -4362,7 +4399,7 @@
       </c>
       <c r="C22" s="18">
         <f>'Таблица для заполнения'!D28</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D22" s="62"/>
       <c r="E22" s="66"/>
@@ -4372,14 +4409,14 @@
       <c r="G22" s="66"/>
       <c r="H22" s="80">
         <f>C22*F22</f>
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="I22" s="80">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J22" s="118"/>
-      <c r="K22" s="119"/>
+        <v>120000</v>
+      </c>
+      <c r="J22" s="119"/>
+      <c r="K22" s="120"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
@@ -4390,14 +4427,14 @@
       </c>
       <c r="C23" s="20">
         <f>'Таблица для заполнения'!D4</f>
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="D23" s="57">
         <v>1000</v>
       </c>
       <c r="E23" s="67">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>90000</v>
       </c>
       <c r="F23" s="57">
         <v>700</v>
@@ -4405,11 +4442,11 @@
       <c r="G23" s="67"/>
       <c r="H23" s="81">
         <f>C23*F23</f>
-        <v>0</v>
+        <v>63000</v>
       </c>
       <c r="I23" s="81">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>153000</v>
       </c>
       <c r="J23" s="117"/>
       <c r="K23" s="117"/>
@@ -4444,8 +4481,8 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J24" s="116"/>
-      <c r="K24" s="116"/>
+      <c r="J24" s="110"/>
+      <c r="K24" s="110"/>
     </row>
     <row r="25" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="21" t="s">
@@ -4456,14 +4493,14 @@
       </c>
       <c r="C25" s="21">
         <f>'Таблица для заполнения'!D30</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D25" s="58">
         <v>28000</v>
       </c>
       <c r="E25" s="68">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>140000</v>
       </c>
       <c r="F25" s="58">
         <v>8000</v>
@@ -4471,14 +4508,14 @@
       <c r="G25" s="68"/>
       <c r="H25" s="82">
         <f>C25*F25</f>
-        <v>0</v>
+        <v>40000</v>
       </c>
       <c r="I25" s="82">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J25" s="120"/>
-      <c r="K25" s="120"/>
+        <v>180000</v>
+      </c>
+      <c r="J25" s="111"/>
+      <c r="K25" s="111"/>
     </row>
     <row r="26" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
@@ -4490,27 +4527,27 @@
       <c r="C26" s="22"/>
       <c r="D26" s="59">
         <f>'Таблица для заполнения'!D31</f>
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="E26" s="69">
         <f>D26</f>
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="F26" s="59">
         <f>'Таблица для заполнения'!D32</f>
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="G26" s="70">
         <f>F26</f>
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="H26" s="69"/>
       <c r="I26" s="78">
         <f>D26+F26</f>
-        <v>0</v>
-      </c>
-      <c r="J26" s="97"/>
-      <c r="K26" s="97"/>
+        <v>100000</v>
+      </c>
+      <c r="J26" s="96"/>
+      <c r="K26" s="96"/>
     </row>
     <row r="27" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
@@ -4521,29 +4558,29 @@
       </c>
       <c r="C27" s="6">
         <f>'Таблица для заполнения'!D33</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D27" s="63">
         <v>6000</v>
       </c>
       <c r="E27" s="51">
         <f>C27*D27</f>
-        <v>0</v>
+        <v>48000</v>
       </c>
       <c r="F27" s="60">
         <v>4000</v>
       </c>
       <c r="G27" s="51">
         <f>C27*F27</f>
-        <v>0</v>
+        <v>32000</v>
       </c>
       <c r="H27" s="78"/>
       <c r="I27" s="78">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J27" s="97"/>
-      <c r="K27" s="97"/>
+        <v>80000</v>
+      </c>
+      <c r="J27" s="96"/>
+      <c r="K27" s="96"/>
     </row>
     <row r="28" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
@@ -4554,30 +4591,30 @@
       </c>
       <c r="C28" s="9">
         <f>'Таблица для заполнения'!D33</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D28" s="59">
         <f>'Таблица для заполнения'!D34</f>
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="E28" s="70">
         <f>D28</f>
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="F28" s="57">
         <v>4000</v>
       </c>
       <c r="G28" s="51">
         <f>C28*F28</f>
-        <v>0</v>
+        <v>32000</v>
       </c>
       <c r="H28" s="78"/>
       <c r="I28" s="78">
         <f>C28*F28+D28</f>
-        <v>0</v>
-      </c>
-      <c r="J28" s="97"/>
-      <c r="K28" s="97"/>
+        <v>152000</v>
+      </c>
+      <c r="J28" s="96"/>
+      <c r="K28" s="96"/>
     </row>
     <row r="29" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
@@ -4588,29 +4625,29 @@
       </c>
       <c r="C29" s="6">
         <f>'Таблица для заполнения'!D35</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D29" s="63">
         <v>12000</v>
       </c>
       <c r="E29" s="51">
         <f>C29*D29</f>
-        <v>0</v>
+        <v>36000</v>
       </c>
       <c r="F29" s="57">
         <v>10000</v>
       </c>
       <c r="G29" s="51">
         <f>C29*F29</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="H29" s="78"/>
       <c r="I29" s="78">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J29" s="97"/>
-      <c r="K29" s="97"/>
+        <v>66000</v>
+      </c>
+      <c r="J29" s="96"/>
+      <c r="K29" s="96"/>
     </row>
     <row r="30" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
@@ -4621,30 +4658,30 @@
       </c>
       <c r="C30" s="9">
         <f>'Таблица для заполнения'!D35</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D30" s="59">
         <f>'Таблица для заполнения'!D36</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="E30" s="70">
         <f>D30</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="F30" s="57">
         <v>10000</v>
       </c>
       <c r="G30" s="51">
         <f>C30*F30</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="H30" s="78"/>
       <c r="I30" s="78">
         <f>D30+F30*C30</f>
-        <v>0</v>
-      </c>
-      <c r="J30" s="97"/>
-      <c r="K30" s="97"/>
+        <v>60000</v>
+      </c>
+      <c r="J30" s="96"/>
+      <c r="K30" s="96"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="23" t="s">
@@ -4655,7 +4692,7 @@
       </c>
       <c r="C31" s="24">
         <f>C1</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D31" s="64"/>
       <c r="E31" s="71"/>
@@ -4665,14 +4702,14 @@
       <c r="G31" s="71"/>
       <c r="H31" s="83">
         <f>C31*F31</f>
-        <v>0</v>
+        <v>204000</v>
       </c>
       <c r="I31" s="83">
         <f>C31*F31</f>
-        <v>0</v>
-      </c>
-      <c r="J31" s="121"/>
-      <c r="K31" s="121"/>
+        <v>204000</v>
+      </c>
+      <c r="J31" s="112"/>
+      <c r="K31" s="112"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="25" t="s">
@@ -4683,14 +4720,14 @@
       </c>
       <c r="C32" s="24">
         <f>C1</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D32" s="57">
         <v>2600</v>
       </c>
       <c r="E32" s="72">
         <f t="shared" ref="E32:E42" si="3">C32*D32</f>
-        <v>0</v>
+        <v>312000</v>
       </c>
       <c r="F32" s="57">
         <v>1800</v>
@@ -4698,14 +4735,14 @@
       <c r="G32" s="72"/>
       <c r="H32" s="84">
         <f>C32*F32</f>
-        <v>0</v>
+        <v>216000</v>
       </c>
       <c r="I32" s="84">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J32" s="122"/>
-      <c r="K32" s="122"/>
+        <v>528000</v>
+      </c>
+      <c r="J32" s="113"/>
+      <c r="K32" s="113"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="26" t="s">
@@ -4716,14 +4753,14 @@
       </c>
       <c r="C33" s="26">
         <f>'Таблица для заполнения'!D37</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D33" s="57">
         <v>60000</v>
       </c>
       <c r="E33" s="73">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>60000</v>
       </c>
       <c r="F33" s="57">
         <f>'Наполнение санузла(вкладка №2)'!L17</f>
@@ -4736,10 +4773,10 @@
       </c>
       <c r="I33" s="85">
         <f>E33+H33</f>
-        <v>82000</v>
-      </c>
-      <c r="J33" s="123"/>
-      <c r="K33" s="123"/>
+        <v>142000</v>
+      </c>
+      <c r="J33" s="114"/>
+      <c r="K33" s="114"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="26" t="s">
@@ -4750,7 +4787,7 @@
       </c>
       <c r="C34" s="26">
         <f>'Таблица для заполнения'!D37</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D34" s="57">
         <f>'Наполнение санузла(вкладка №2)'!E24</f>
@@ -4758,17 +4795,17 @@
       </c>
       <c r="E34" s="73">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>205000</v>
       </c>
       <c r="F34" s="61"/>
       <c r="G34" s="73"/>
       <c r="H34" s="85"/>
       <c r="I34" s="85">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J34" s="124"/>
-      <c r="K34" s="125"/>
+        <v>205000</v>
+      </c>
+      <c r="J34" s="115"/>
+      <c r="K34" s="116"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
@@ -4779,29 +4816,29 @@
       </c>
       <c r="C35" s="24">
         <f>C1</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D35" s="57">
         <v>600</v>
       </c>
       <c r="E35" s="51">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>72000</v>
       </c>
       <c r="F35" s="57">
         <v>100</v>
       </c>
       <c r="G35" s="51">
         <f>C35*F35</f>
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="H35" s="9"/>
       <c r="I35" s="78">
         <f>(D35+F35)*C35</f>
-        <v>0</v>
-      </c>
-      <c r="J35" s="98"/>
-      <c r="K35" s="99"/>
+        <v>84000</v>
+      </c>
+      <c r="J35" s="97"/>
+      <c r="K35" s="98"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
@@ -4812,24 +4849,24 @@
       </c>
       <c r="C36" s="24">
         <f>C1</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D36" s="57">
         <v>1600</v>
       </c>
       <c r="E36" s="51">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>192000</v>
       </c>
       <c r="F36" s="27"/>
       <c r="G36" s="76"/>
       <c r="H36" s="28"/>
       <c r="I36" s="51">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J36" s="97"/>
-      <c r="K36" s="97"/>
+        <v>192000</v>
+      </c>
+      <c r="J36" s="96"/>
+      <c r="K36" s="96"/>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
@@ -4840,24 +4877,24 @@
       </c>
       <c r="C37" s="24">
         <f>C1</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D37" s="57">
         <v>600</v>
       </c>
       <c r="E37" s="51">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>72000</v>
       </c>
       <c r="F37" s="19"/>
       <c r="G37" s="51"/>
       <c r="H37" s="6"/>
       <c r="I37" s="51">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J37" s="97"/>
-      <c r="K37" s="97"/>
+        <v>72000</v>
+      </c>
+      <c r="J37" s="96"/>
+      <c r="K37" s="96"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="6"/>
@@ -4878,8 +4915,8 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J38" s="97"/>
-      <c r="K38" s="97"/>
+      <c r="J38" s="96"/>
+      <c r="K38" s="96"/>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="6"/>
@@ -4900,8 +4937,8 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J39" s="97"/>
-      <c r="K39" s="97"/>
+      <c r="J39" s="96"/>
+      <c r="K39" s="96"/>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="6"/>
@@ -4922,8 +4959,8 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J40" s="97"/>
-      <c r="K40" s="97"/>
+      <c r="J40" s="96"/>
+      <c r="K40" s="96"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="6"/>
@@ -4944,8 +4981,8 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J41" s="97"/>
-      <c r="K41" s="97"/>
+      <c r="J41" s="96"/>
+      <c r="K41" s="96"/>
     </row>
     <row r="42" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="29"/>
@@ -4966,8 +5003,8 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J42" s="126"/>
-      <c r="K42" s="126"/>
+      <c r="J42" s="105"/>
+      <c r="K42" s="105"/>
     </row>
     <row r="43" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="30" t="s">
@@ -4978,7 +5015,7 @@
       </c>
       <c r="C43" s="32">
         <f>C1</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D43" s="75">
         <v>13500</v>
@@ -4989,10 +5026,10 @@
       <c r="H43" s="31"/>
       <c r="I43" s="86">
         <f>D43*C43</f>
-        <v>0</v>
-      </c>
-      <c r="J43" s="127"/>
-      <c r="K43" s="128"/>
+        <v>1620000</v>
+      </c>
+      <c r="J43" s="106"/>
+      <c r="K43" s="107"/>
     </row>
     <row r="44" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I44" s="87"/>
@@ -5006,23 +5043,23 @@
       <c r="D45" s="34"/>
       <c r="E45" s="77">
         <f>SUM(E6:E43)</f>
-        <v>0</v>
+        <v>6489475</v>
       </c>
       <c r="F45" s="34"/>
       <c r="G45" s="77">
         <f>SUM(G6:G43)</f>
-        <v>0</v>
+        <v>1912500</v>
       </c>
       <c r="H45" s="77">
         <f>SUM(H4:H42)</f>
-        <v>82000</v>
+        <v>825000</v>
       </c>
       <c r="I45" s="77">
         <f>SUM(I4:I42)+I43</f>
-        <v>82000</v>
-      </c>
-      <c r="J45" s="129"/>
-      <c r="K45" s="106"/>
+        <v>11321075</v>
+      </c>
+      <c r="J45" s="108"/>
+      <c r="K45" s="109"/>
     </row>
     <row r="46" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I46" s="87"/>
@@ -5040,7 +5077,7 @@
       <c r="H47" s="36"/>
       <c r="I47" s="88">
         <f>I45*1.38</f>
-        <v>113159.99999999999</v>
+        <v>15623083.499999998</v>
       </c>
       <c r="J47" s="36"/>
       <c r="K47" s="37"/>
@@ -5232,39 +5269,6 @@
     </row>
   </sheetData>
   <mergeCells count="46">
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="J43:K43"/>
-    <mergeCell ref="J45:K45"/>
-    <mergeCell ref="J36:K36"/>
-    <mergeCell ref="J37:K37"/>
-    <mergeCell ref="J38:K38"/>
-    <mergeCell ref="J39:K39"/>
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="J41:K41"/>
-    <mergeCell ref="J35:K35"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
     <mergeCell ref="J10:K10"/>
     <mergeCell ref="N10:O10"/>
     <mergeCell ref="A1:A2"/>
@@ -5278,6 +5282,39 @@
     <mergeCell ref="J8:K8"/>
     <mergeCell ref="N8:O8"/>
     <mergeCell ref="J9:K9"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="J43:K43"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="J39:K39"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="J41:K41"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>